<commit_message>
added AI visual feature + version number
</commit_message>
<xml_diff>
--- a/uploads/esempioReale_corretto.xlsx
+++ b/uploads/esempioReale_corretto.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Viale De Gasperi, 69, Avio, Trento, Italy</t>
+          <t>Viale Alcide Degasperi, 69, Avio, Trento, Italy</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -603,7 +603,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Piazzale Stazione, Mezzolombardo, Trento, Italy</t>
+          <t>Via della Stazione, Mezzolombardo, Trento, Italy</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -622,7 +622,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Via Spiazzi, 2, Zivignago, Trento, Italy</t>
+          <t>Via Spiazzi, 2, Pergine Valsugana, Trento, Italy</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Corso De Gasperi, 8, Predazzo, Trento, Italy</t>
+          <t>Corso Alcide Degasperi, 8, Predazzo, Trento, Italy</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -725,7 +725,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Via Roma, Ospedaletto, Trento, Italy</t>
+          <t>Via Roma, Castel Ivano, Trento, Italy</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Via Alcide De Gasperi, 5, 38096, Terlago, Trento, Italy</t>
+          <t>Via Alcide Degasperi, 5, 38096, Terlago, Trento, Italy</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -763,7 +763,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Piazza de Ciampiedel, Campitello di Fassa, Trento, Italy</t>
+          <t>Piazza Gries, Canazei, Trento, Italy</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Piazza de Ciampiedel, Campitello di Fassa, Trento, Italy</t>
+          <t>Piazza, Campitello di Fassa, Trento, Italy</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Via della Credenza, Taio, Trento, Italy</t>
+          <t>Via Giovanni Segantini, Taio, Trento, Italy</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Trento, Trento, Italy</t>
+          <t>Via Sant'Anna, 6, 38121, Trento, Trento, Italy</t>
         </is>
       </c>
       <c r="C23" t="n">

</xml_diff>

<commit_message>
added google maps + AI tool
</commit_message>
<xml_diff>
--- a/uploads/esempioReale_corretto.xlsx
+++ b/uploads/esempioReale_corretto.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Piazza Condini, Romagnano, Trento, Italy</t>
+          <t>Piazza Condini, Romagnano</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Via del Comun, 8, Commezzadura, Trento, Italy</t>
+          <t>Via del Comun, 8, Commezzadura</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Viale Degasperi, 69, Avio, Trento, Italy</t>
+          <t>Viale Alcide Degasperi, 69, Avio</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -508,7 +508,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Via 24 Maggio, 115, Lodrone, Trento, Italy</t>
+          <t>Via 24 Maggio, 115, Lodrone</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -527,7 +527,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Strada Provinciale di Seregnano, 4, Cogatti, Trento, Italy</t>
+          <t>Frazione Cogatti, 4, Seregnano</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Piazza Fiera, Cles, Trento, Italy</t>
+          <t>Piazza Fiera, Cles</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -565,7 +565,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Balbido, 1, 38071, Bleggio Superiore, Trento, Italy</t>
+          <t>Frazione Balbido, 1, Bleggio Superiore</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -584,7 +584,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Via Biasi, 1, 38010, San Michele all'Adige, Trento, Italy</t>
+          <t>Via Biasi, 1, San Michele all'Adige</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -603,7 +603,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Piazzale della Stazione, Mezzolombardo, Trento, Italy</t>
+          <t>Mezzolombardo Stazione FTM, Mezzolombardo</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -622,7 +622,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Via Spiazzi, 2, Zivignago, Trento, Italy</t>
+          <t>Via Spiazzi, 2, Canezza</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Corso Degasperi, 8, Predazzo, Trento, Italy</t>
+          <t>Corso de Gasperi, 8, Predazzo</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -660,7 +660,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Via Sant'Alessandro, 11, Riva del Garda, Trento, Italy</t>
+          <t>Via S. Alessandro, 11, Riva del Garda</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Via dei Laghi, 47, 38060, Tenno, Trento, Italy</t>
+          <t>Via dei Laghi, 47, Tenno</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Viale Trento, Rovereto, Trento, Italy</t>
+          <t>Viale Trento, Rovereto</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -725,7 +725,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Via Roma, Spedaletto, Trento, Italy</t>
+          <t>Via Roma, Ospedaletto</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Via Alcide Degasperi, 5, 38096, Terlago, Trento, Italy</t>
+          <t>Via Alcide Degasperi, 5, Terlago</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -763,7 +763,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gries, Canazei, Trento, Italy</t>
+          <t>Gries, Canazei</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -782,7 +782,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Via Temanza, Borgo Valsugana, Trento, Italy</t>
+          <t>Via Temanza, Borgo Valsugana</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Piazza de Ciampedel, Campitello di Fassa, Trento, Italy</t>
+          <t>Piazza Centrale, Campitello di Fassa</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Via Albere, 2, Tenna, Trento, Italy</t>
+          <t>Via Alberè, 2, Tenna</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Via Guglielmo Marconi, Taio, Trento, Italy</t>
+          <t>Taio, Predaia</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Corso Tre Novembre, 132, 38122, Trento, Trento, Italy</t>
+          <t>Via IV Novembre, Trento</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -877,7 +877,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Via Alessandro Manzoni, 3, 38068, Rovereto, Trento, Italy</t>
+          <t>Via Alessandro Manzoni, 3, Rovereto</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>

</xml_diff>

<commit_message>
resolved part of maps problems
</commit_message>
<xml_diff>
--- a/uploads/esempioReale_corretto.xlsx
+++ b/uploads/esempioReale_corretto.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Piazza Condini, Romagnano</t>
+          <t>Piazza Costantino Condini, Romagnano, Trento, TN, Italia</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Via del Comun, 8, Commezzadura</t>
+          <t>Via del Comun, 8, Commezzadura, TN, Italia</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Viale Alcide Degasperi, 69, Avio</t>
+          <t>Viale Alcide Degasperi, 69, Avio, TN, Italia</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -508,7 +508,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Via 24 Maggio, 115, Lodrone</t>
+          <t>Via 24 Maggio, 115, Lodrone, Storo, TN, Italia</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -527,7 +527,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Frazione Cogatti, 4, Seregnano</t>
+          <t>Frazione Cogatti, 4, Seregnano, Civezzano, TN, Italia</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Piazza Fiera, Cles</t>
+          <t>Piazza Fiera, Cles, TN, Italia</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -565,7 +565,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Frazione Balbido, 1, Bleggio Superiore</t>
+          <t>Frazione Balbido, 1, Bleggio Superiore, TN, Italia</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -584,7 +584,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Via Biasi, 1, San Michele all'Adige</t>
+          <t>Via Biasi, 1, San Michele all'Adige, TN, Italia</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -603,7 +603,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mezzolombardo Stazione FTM, Mezzolombardo</t>
+          <t>Mezzolombardo Stazione FTM, Mezzolombardo, TN, Italia</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -622,7 +622,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Via Spiazzi, 2, Canezza</t>
+          <t>Via Spiazzi, 2, Pergine Valsugana, TN, Italia</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Corso de Gasperi, 8, Predazzo</t>
+          <t>Corso de Gasperi, 8, Predazzo, TN, Italia</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -660,7 +660,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Via S. Alessandro, 11, Riva del Garda</t>
+          <t>Via S. Alessandro, 11, Riva del Garda, TN, Italia</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Via dei Laghi, 47, Tenno</t>
+          <t>Via dei Laghi, 47, Tenno, TN, Italia</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Viale Trento, Rovereto</t>
+          <t>Viale Trento, Rovereto, TN, Italia</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -725,7 +725,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Via Roma, Ospedaletto</t>
+          <t>Via Roma, Ospedaletto, TN, Italia</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Via Alcide Degasperi, 5, Terlago</t>
+          <t>Via Alcide Degasperi, 5, Vallelaghi, TN, Italia</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -763,7 +763,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gries, Canazei</t>
+          <t>Canazei. Gries, Canazei, TN, Italia</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -782,7 +782,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Via Temanza, Borgo Valsugana</t>
+          <t>Via Temanza, Borgo Valsugana, TN, Italia</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Piazza Centrale, Campitello di Fassa</t>
+          <t>Piazza Centrale, Campitello di Fassa, TN, Italia</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Via Alberè, 2, Tenna</t>
+          <t>Via Alberè, 2, Tenna, TN, Italia</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Taio, Predaia</t>
+          <t>Taio, Predaia, TN, Italia</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Via IV Novembre, Trento</t>
+          <t>Via IV Novembre, Trento, TN, Italia</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -877,7 +877,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Via Alessandro Manzoni, 3, Rovereto</t>
+          <t>Via Alessandro Manzoni, 3, Rovereto, TN, Italia</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>

</xml_diff>

<commit_message>
ADDEDD ALL FEATURES (need to fix a thing)
</commit_message>
<xml_diff>
--- a/uploads/esempioReale_corretto.xlsx
+++ b/uploads/esempioReale_corretto.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Romagnano Piazza Condini, Romagnano, TN, Italia</t>
+          <t>Piazza Costantino Condini, Romagnano, Trento, TN</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Via del Comun, 8, Commezzadura, TN, Italia</t>
+          <t>Via del Comun, 8, Commezzadura, TN</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Viale Alcide Degasperi, 69, Avio, TN, Italia</t>
+          <t>Viale Alcide Degasperi, 69, Avio, TN</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -508,7 +508,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Via 24 Maggio, 115, Lodrone, TN, Italia</t>
+          <t>Via 24 Maggio, 115, Lodrone, TN</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -527,7 +527,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Frazione Cogatti, 4, Seregnano, TN, Italia</t>
+          <t>Frazione Cogatti, 4, Seregnano, TN</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Piazza Fiera, Cles, TN, Italia</t>
+          <t>Piazza Fiera, Cles, TN</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -565,7 +565,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Località Balbido, 1, Bleggio Superiore, TN, Italia</t>
+          <t>Frazione Balbido, 1, Bleggio Superiore, TN</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -584,7 +584,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Via Biasi, 1, San Michele all'Adige, TN, Italia</t>
+          <t>Via Biasi, 1, San Michele all'Adige, TN</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -603,7 +603,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mezzolombardo Stazione FTM, Mezzolombardo, TN, Italia</t>
+          <t>Mezzolombardo Stazione FTM, Mezzolombardo, TN</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -622,7 +622,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Via Spiazzi, 2, Canezza, Pergine Valsugana, TN, Italia</t>
+          <t>Via Spiazzi, 2, Canezza, Pergine Valsugana, TN</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Corso de Gasperi, 8, Predazzo, TN, Italia</t>
+          <t>Corso de Gasperi, 8, Predazzo, TN</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -660,7 +660,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Via S. Alessandro, 11, Riva del Garda, TN, Italia</t>
+          <t>Via S. Alessandro, 11, Riva del Garda, TN</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Via dei Laghi, 47, Tenno, TN, Italia</t>
+          <t>Via dei Laghi, 47, Tenno, TN</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Viale Trento, Rovereto, TN, Italia</t>
+          <t>Viale Trento, Rovereto, TN</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -725,7 +725,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Via Roma, Ospedaletto, TN, Italia</t>
+          <t>Via Roma, Ospedaletto, TN</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Via Alcide Degasperi, 5, Vallelaghi, TN, Italia</t>
+          <t>Via Alcide De Gasperi, 5, Vallelaghi, TN</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -763,7 +763,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Piazza Gries, Canazei, TN, Italia</t>
+          <t>Gries, Canazei, TN</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -782,7 +782,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Via Temanza, Borgo Valsugana, TN, Italia</t>
+          <t>Via Temanza, Borgo Valsugana, TN</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Piazza Centrale, Campitello di Fassa, TN, Italia</t>
+          <t>Piazza Centrale, Campitello di Fassa, TN</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Via Alberè, 2, Tenna, TN, Italia</t>
+          <t>Via Alberè, 2, Tenna, TN</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Taio, Predaia, TN, Italia</t>
+          <t>Taio, Predaia, TN</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Via Alessandro Manzoni, 3, Rovereto, TN, Italia</t>
+          <t>Via Alessandro Manzoni, 3, Rovereto, TN</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>

<commit_message>
ADDED ALL FEATURES REQUIRED and fixed firebase
</commit_message>
<xml_diff>
--- a/uploads/esempioReale_corretto.xlsx
+++ b/uploads/esempioReale_corretto.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Piazza Costantino Condini, Romagnano, Trento, TN</t>
+          <t>Piazza Costantino Condini, Romagnano, Trento, TN, Italia</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Via del Comun, 8, Commezzadura, TN</t>
+          <t>Via del Comun, 8, Commezzadura, TN, Italia</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Viale Alcide Degasperi, 69, Avio, TN</t>
+          <t>Viale Alcide Degasperi, 69, Avio, TN, Italia</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -508,7 +508,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Via 24 Maggio, 115, Lodrone, TN</t>
+          <t>Via 24 Maggio, 115, Lodrone, Storo, TN, Italia</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -527,7 +527,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Frazione Cogatti, 4, Seregnano, TN</t>
+          <t>Frazione Cogatti, 4, Seregnano, Civezzano, TN, Italia</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Piazza Fiera, Cles, TN</t>
+          <t>Piazza Fiera, Cles, TN, Italia</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -565,7 +565,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Frazione Balbido, 1, Bleggio Superiore, TN</t>
+          <t>Località Balbido, 1, Bleggio Superiore, TN, Italia</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -584,7 +584,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Via Biasi, 1, San Michele all'Adige, TN</t>
+          <t>Via Biasi, 1, San Michele all'Adige, TN, Italia</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -603,7 +603,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mezzolombardo Stazione FTM, Mezzolombardo, TN</t>
+          <t>Mezzolombardo Stazione FTM, Mezzolombardo, TN, Italia</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -622,7 +622,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Via Spiazzi, 2, Canezza, Pergine Valsugana, TN</t>
+          <t>Via Spiazzi, 2, Canezza, Pergine Valsugana, TN, Italia</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Corso de Gasperi, 8, Predazzo, TN</t>
+          <t>Corso de Gasperi, 8, Predazzo, TN, Italia</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -660,7 +660,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Via S. Alessandro, 11, Riva del Garda, TN</t>
+          <t>Via S.Alessandro, 11, Riva del Garda, TN, Italia</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Via dei Laghi, 47, Tenno, TN</t>
+          <t>Via dei Laghi, 47, Tenno, TN, Italia</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Viale Trento, Rovereto, TN</t>
+          <t>Viale Trento, Rovereto, TN, Italia</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -725,7 +725,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Via Roma, Ospedaletto, TN</t>
+          <t>Via Roma, Spera, Castel Ivano, TN, Italia</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Via Alcide De Gasperi, 5, Vallelaghi, TN</t>
+          <t>Via Alcide De Gasperi, 5, Vallelaghi, TN, Italia</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -763,7 +763,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gries, Canazei, TN</t>
+          <t>Gries, Canazei, TN, Italia</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -782,7 +782,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Via Temanza, Borgo Valsugana, TN</t>
+          <t>Via Temanza, Borgo Valsugana, TN, Italia</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Piazza Centrale, Campitello di Fassa, TN</t>
+          <t>Piazza Centrale, Campitello di Fassa, TN, Italia</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Via Alberè, 2, Tenna, TN</t>
+          <t>Via Alberè, 2, Tenna, TN, Italia</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Taio, Predaia, TN</t>
+          <t>Via Giovanni a Prato, 1, Taio, Predaia, TN, Italia</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Via Alessandro Manzoni, 3, Rovereto, TN</t>
+          <t>Via Alessandro Manzoni, 3, Rovereto, TN, Italia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>